<commit_message>
In leads_steps new scenario of updating the created lead data is implemented.In the excel sheet new test data is added.In leads featuire file sceanrio is added
</commit_message>
<xml_diff>
--- a/Data/Testdata.xlsx
+++ b/Data/Testdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\PycharmProjects\Behave framework\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3CB121C-2150-4CB6-A58F-1FA5CDE4A33F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03FF8D19-C3DB-41DE-BAD7-E9699A230A2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
   <si>
     <t>ScenarioName</t>
   </si>
@@ -61,6 +61,18 @@
   </si>
   <si>
     <t>NDA</t>
+  </si>
+  <si>
+    <t>admin456</t>
+  </si>
+  <si>
+    <t>Edit_existing_lead_TC05</t>
+  </si>
+  <si>
+    <t>sitaraman</t>
+  </si>
+  <si>
+    <t>UPA</t>
   </si>
 </sst>
 </file>
@@ -90,7 +102,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -113,14 +125,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -401,7 +425,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="48.33203125" customWidth="1"/>
@@ -444,8 +468,8 @@
       <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="1">
-        <v>3243253</v>
+      <c r="C3" s="1" t="s">
+        <v>12</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -467,6 +491,17 @@
         <v>11</v>
       </c>
     </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>